<commit_message>
Update past-year DSM-IV diagnosed substance abuse disorder in AddictO_Human-being_Defs.xlsx
</commit_message>
<xml_diff>
--- a/inputs/AddictO_Human-being_Defs.xlsx
+++ b/inputs/AddictO_Human-being_Defs.xlsx
@@ -19744,25 +19744,14 @@
           <t>mental disposition</t>
         </is>
       </c>
-      <c r="E365" t="inlineStr"/>
-      <c r="F365" t="inlineStr"/>
       <c r="G365" t="inlineStr">
         <is>
           <t>Human being</t>
         </is>
       </c>
-      <c r="H365" t="inlineStr"/>
-      <c r="I365" t="inlineStr"/>
-      <c r="J365" t="inlineStr"/>
-      <c r="K365" t="inlineStr"/>
       <c r="L365" t="n">
         <v>0</v>
       </c>
-      <c r="M365" t="inlineStr"/>
-      <c r="N365" t="inlineStr"/>
-      <c r="O365" t="inlineStr"/>
-      <c r="P365" t="inlineStr"/>
-      <c r="Q365" t="inlineStr"/>
       <c r="R365" t="inlineStr">
         <is>
           <t>disposition</t>
@@ -19776,7 +19765,6 @@
       <c r="T365" t="n">
         <v>0</v>
       </c>
-      <c r="U365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -26407,47 +26395,47 @@
       <c r="U494" s="3" t="n"/>
     </row>
     <row r="495">
-      <c r="A495" s="4" t="n"/>
-      <c r="B495" s="4" t="inlineStr">
+      <c r="A495" s="3" t="n"/>
+      <c r="B495" s="3" t="inlineStr">
         <is>
           <t>past-year DSM-IV diagnosed substance abuse disorder</t>
         </is>
       </c>
-      <c r="C495" s="4" t="n"/>
-      <c r="D495" s="4" t="n"/>
-      <c r="E495" s="4" t="n"/>
-      <c r="F495" s="4" t="n"/>
-      <c r="G495" s="4" t="inlineStr">
-        <is>
-          <t>Human being</t>
-        </is>
-      </c>
-      <c r="H495" s="4" t="n"/>
-      <c r="I495" s="4" t="n"/>
-      <c r="J495" s="4" t="n"/>
-      <c r="K495" s="4" t="n"/>
-      <c r="L495" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M495" s="4" t="n"/>
-      <c r="N495" s="4" t="n"/>
-      <c r="O495" s="4" t="n"/>
-      <c r="P495" s="4" t="n"/>
-      <c r="Q495" s="4" t="n"/>
-      <c r="R495" s="4" t="n"/>
-      <c r="S495" s="4" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="T495" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U495" s="4" t="n"/>
+      <c r="C495" s="3" t="n"/>
+      <c r="D495" s="3" t="n"/>
+      <c r="E495" s="3" t="n"/>
+      <c r="F495" s="3" t="n"/>
+      <c r="G495" s="3" t="inlineStr">
+        <is>
+          <t>Human being</t>
+        </is>
+      </c>
+      <c r="H495" s="3" t="n"/>
+      <c r="I495" s="3" t="n"/>
+      <c r="J495" s="3" t="n"/>
+      <c r="K495" s="3" t="n"/>
+      <c r="L495" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M495" s="3" t="n"/>
+      <c r="N495" s="3" t="n"/>
+      <c r="O495" s="3" t="n"/>
+      <c r="P495" s="3" t="n"/>
+      <c r="Q495" s="3" t="n"/>
+      <c r="R495" s="3" t="n"/>
+      <c r="S495" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="T495" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U495" s="3" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update past-year DSM diagnosed substance use disorder in AddictO_Human-being_Defs.xlsx
</commit_message>
<xml_diff>
--- a/inputs/AddictO_Human-being_Defs.xlsx
+++ b/inputs/AddictO_Human-being_Defs.xlsx
@@ -26395,47 +26395,67 @@
       <c r="U494" s="3" t="n"/>
     </row>
     <row r="495">
-      <c r="A495" s="4" t="n"/>
-      <c r="B495" s="4" t="inlineStr">
-        <is>
-          <t>past-year DSM-IV diagnosed substance abuse disorder</t>
-        </is>
-      </c>
-      <c r="C495" s="4" t="n"/>
-      <c r="D495" s="4" t="n"/>
-      <c r="E495" s="4" t="n"/>
-      <c r="F495" s="4" t="n"/>
-      <c r="G495" s="4" t="inlineStr">
-        <is>
-          <t>Human being</t>
-        </is>
-      </c>
-      <c r="H495" s="4" t="n"/>
-      <c r="I495" s="4" t="n"/>
-      <c r="J495" s="4" t="n"/>
-      <c r="K495" s="4" t="n"/>
-      <c r="L495" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M495" s="4" t="n"/>
-      <c r="N495" s="4" t="n"/>
-      <c r="O495" s="4" t="n"/>
-      <c r="P495" s="4" t="n"/>
-      <c r="Q495" s="4" t="n"/>
-      <c r="R495" s="4" t="n"/>
-      <c r="S495" s="4" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="T495" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U495" s="4" t="n"/>
+      <c r="A495" s="3" t="inlineStr">
+        <is>
+          <t>ADDICTO:0001431</t>
+        </is>
+      </c>
+      <c r="B495" s="3" t="inlineStr">
+        <is>
+          <t>past-year DSM diagnosed substance use disorder</t>
+        </is>
+      </c>
+      <c r="C495" s="3" t="inlineStr">
+        <is>
+          <t>A personal attribute that involves the person having received a diagnosis of substance use disorder in the past 12 months using DSM criteria.</t>
+        </is>
+      </c>
+      <c r="D495" s="3" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
+      <c r="E495" s="3" t="n"/>
+      <c r="F495" s="3" t="inlineStr">
+        <is>
+          <t>The class is used for diagnosis of any edition of DSM to maintain continuity as new editions are created.</t>
+        </is>
+      </c>
+      <c r="G495" s="3" t="inlineStr">
+        <is>
+          <t>Human being</t>
+        </is>
+      </c>
+      <c r="H495" s="3" t="inlineStr"/>
+      <c r="I495" s="3" t="n"/>
+      <c r="J495" s="3" t="n"/>
+      <c r="K495" s="3" t="n"/>
+      <c r="L495" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M495" s="3" t="n"/>
+      <c r="N495" s="3" t="n"/>
+      <c r="O495" s="3" t="n"/>
+      <c r="P495" s="3" t="n"/>
+      <c r="Q495" s="3" t="n"/>
+      <c r="R495" s="3" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+      <c r="S495" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="T495" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U495" s="3" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update 2 terms in AddictO_Human-being_Defs.xlsx
</commit_message>
<xml_diff>
--- a/inputs/AddictO_Human-being_Defs.xlsx
+++ b/inputs/AddictO_Human-being_Defs.xlsx
@@ -26418,7 +26418,7 @@
       <c r="E495" s="3" t="n"/>
       <c r="F495" s="3" t="inlineStr">
         <is>
-          <t>The class is used for diagnosis of any edition of DSM to maintain continuity as new editions are created.</t>
+          <t>The class is used for diagnosis of any edition of DSM to maintain continuity as new editions are created. It is a personal attribute because the focus is on the mental health of the person rather, with the diagnosis being an indicator of that health.</t>
         </is>
       </c>
       <c r="G495" s="3" t="inlineStr">
@@ -26426,7 +26426,7 @@
           <t>Human being</t>
         </is>
       </c>
-      <c r="H495" s="3" t="inlineStr"/>
+      <c r="H495" s="3" t="n"/>
       <c r="I495" s="3" t="n"/>
       <c r="J495" s="3" t="n"/>
       <c r="K495" s="3" t="n"/>
@@ -26538,7 +26538,12 @@
         </is>
       </c>
       <c r="E497" s="3" t="n"/>
-      <c r="F497" s="3" t="n"/>
+      <c r="F497" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is a personal history part because the focus is on the activity of advice which is a process, rather than an attribute of the person.
+</t>
+        </is>
+      </c>
       <c r="G497" s="3" t="inlineStr">
         <is>
           <t>Human being</t>

</xml_diff>

<commit_message>
Update Parent of ever tobacco smoker  in AddictO_Human-being_Defs.xlsx
</commit_message>
<xml_diff>
--- a/inputs/AddictO_Human-being_Defs.xlsx
+++ b/inputs/AddictO_Human-being_Defs.xlsx
@@ -13327,7 +13327,7 @@
       </c>
       <c r="D240" s="3" t="inlineStr">
         <is>
-          <t>tobacco smoker</t>
+          <t>person</t>
         </is>
       </c>
       <c r="E240" s="3" t="inlineStr">
@@ -22959,7 +22959,7 @@
         </is>
       </c>
       <c r="H429" s="3" t="n"/>
-      <c r="I429" s="3" t="inlineStr"/>
+      <c r="I429" s="3" t="n"/>
       <c r="J429" s="3" t="n"/>
       <c r="K429" s="3" t="inlineStr">
         <is>

</xml_diff>